<commit_message>
Add 2023 to GGGI data
</commit_message>
<xml_diff>
--- a/data/GGGI.xlsx
+++ b/data/GGGI.xlsx
@@ -462,7 +462,7 @@
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>GGGI_2002_2022_avg</t>
+          <t>GGGI_2002_2023_avg</t>
         </is>
       </c>
     </row>
@@ -537,7 +537,7 @@
         </is>
       </c>
       <c r="V2">
-        <v>0.7042705882352941</v>
+        <v>0.7085</v>
       </c>
     </row>
     <row r="3">
@@ -611,7 +611,7 @@
         </is>
       </c>
       <c r="V3">
-        <v>0.6138235294117647</v>
+        <v>0.6137111111111111</v>
       </c>
     </row>
     <row r="4">
@@ -682,7 +682,7 @@
         </is>
       </c>
       <c r="V4">
-        <v>0.640025</v>
+        <v>0.6416705882352941</v>
       </c>
     </row>
     <row r="5">
@@ -756,7 +756,7 @@
         </is>
       </c>
       <c r="V5">
-        <v>0.7287176470588236</v>
+        <v>0.7311055555555556</v>
       </c>
     </row>
     <row r="6">
@@ -830,7 +830,7 @@
         </is>
       </c>
       <c r="V6">
-        <v>0.7322882352941177</v>
+        <v>0.7349333333333333</v>
       </c>
     </row>
     <row r="7">
@@ -904,7 +904,7 @@
         </is>
       </c>
       <c r="V7">
-        <v>0.7280529411764706</v>
+        <v>0.7289</v>
       </c>
     </row>
     <row r="8">
@@ -978,7 +978,7 @@
         </is>
       </c>
       <c r="V8">
-        <v>0.6235470588235295</v>
+        <v>0.6259055555555556</v>
       </c>
     </row>
     <row r="9">
@@ -1052,7 +1052,7 @@
         </is>
       </c>
       <c r="V9">
-        <v>0.6876176470588236</v>
+        <v>0.6876944444444444</v>
       </c>
     </row>
     <row r="10">
@@ -1126,7 +1126,7 @@
         </is>
       </c>
       <c r="V10">
-        <v>0.7518823529411764</v>
+        <v>0.7541666666666667</v>
       </c>
     </row>
     <row r="11">
@@ -1200,7 +1200,7 @@
         </is>
       </c>
       <c r="V11">
-        <v>0.7100705882352941</v>
+        <v>0.7120666666666666</v>
       </c>
     </row>
     <row r="12">
@@ -1274,7 +1274,7 @@
         </is>
       </c>
       <c r="V12">
-        <v>0.7009823529411765</v>
+        <v>0.7026166666666667</v>
       </c>
     </row>
     <row r="13">
@@ -1348,7 +1348,7 @@
         </is>
       </c>
       <c r="V13">
-        <v>0.683635294117647</v>
+        <v>0.6854166666666667</v>
       </c>
     </row>
     <row r="14">
@@ -1422,7 +1422,7 @@
         </is>
       </c>
       <c r="V14">
-        <v>0.7206176470588235</v>
+        <v>0.7207722222222223</v>
       </c>
     </row>
     <row r="15">
@@ -1496,7 +1496,7 @@
         </is>
       </c>
       <c r="V15">
-        <v>0.6610823529411765</v>
+        <v>0.6624333333333333</v>
       </c>
     </row>
     <row r="16">
@@ -1567,7 +1567,7 @@
         </is>
       </c>
       <c r="V16">
-        <v>0.6516125</v>
+        <v>0.6540705882352941</v>
       </c>
     </row>
     <row r="17">
@@ -1641,7 +1641,7 @@
         </is>
       </c>
       <c r="V17">
-        <v>0.7453705882352941</v>
+        <v>0.7462277777777778</v>
       </c>
     </row>
     <row r="18">
@@ -1715,7 +1715,7 @@
         </is>
       </c>
       <c r="V18">
-        <v>0.6987411764705882</v>
+        <v>0.6961888888888889</v>
       </c>
     </row>
     <row r="19">
@@ -1789,7 +1789,7 @@
         </is>
       </c>
       <c r="V19">
-        <v>0.5619588235294117</v>
+        <v>0.5627444444444445</v>
       </c>
     </row>
     <row r="20">
@@ -1863,7 +1863,7 @@
         </is>
       </c>
       <c r="V20">
-        <v>0.6982647058823529</v>
+        <v>0.7028666666666666</v>
       </c>
     </row>
     <row r="21">
@@ -1937,7 +1937,7 @@
         </is>
       </c>
       <c r="V21">
-        <v>0.6796647058823529</v>
+        <v>0.6798777777777778</v>
       </c>
     </row>
     <row r="22">
@@ -2011,7 +2011,7 @@
         </is>
       </c>
       <c r="V22">
-        <v>0.7141999999999999</v>
+        <v>0.7159388888888889</v>
       </c>
     </row>
     <row r="23">
@@ -2085,7 +2085,7 @@
         </is>
       </c>
       <c r="V23">
-        <v>0.7372882352941177</v>
+        <v>0.73995</v>
       </c>
     </row>
     <row r="24">
@@ -2156,7 +2156,7 @@
         </is>
       </c>
       <c r="V24">
-        <v>0.7096749999999999</v>
+        <v>0.7104588235294118</v>
       </c>
     </row>
     <row r="25">
@@ -2230,7 +2230,7 @@
         </is>
       </c>
       <c r="V25">
-        <v>0.6752823529411764</v>
+        <v>0.6769555555555555</v>
       </c>
     </row>
     <row r="26">
@@ -2304,7 +2304,7 @@
         </is>
       </c>
       <c r="V26">
-        <v>0.6859235294117647</v>
+        <v>0.6858111111111111</v>
       </c>
     </row>
     <row r="27">
@@ -2375,7 +2375,7 @@
         </is>
       </c>
       <c r="V27">
-        <v>0.6087875</v>
+        <v>0.6099882352941176</v>
       </c>
     </row>
     <row r="28">
@@ -2449,7 +2449,7 @@
         </is>
       </c>
       <c r="V28">
-        <v>0.770035294117647</v>
+        <v>0.7710722222222223</v>
       </c>
     </row>
     <row r="29">
@@ -2523,7 +2523,7 @@
         </is>
       </c>
       <c r="V29">
-        <v>0.6853058823529412</v>
+        <v>0.6864833333333333</v>
       </c>
     </row>
     <row r="30">
@@ -2597,7 +2597,7 @@
         </is>
       </c>
       <c r="V30">
-        <v>0.7201882352941177</v>
+        <v>0.7239722222222222</v>
       </c>
     </row>
     <row r="31">
@@ -2671,7 +2671,7 @@
         </is>
       </c>
       <c r="V31">
-        <v>0.6920235294117647</v>
+        <v>0.6921944444444444</v>
       </c>
     </row>
     <row r="32">
@@ -2745,7 +2745,7 @@
         </is>
       </c>
       <c r="V32">
-        <v>0.6397647058823529</v>
+        <v>0.6435999999999999</v>
       </c>
     </row>
     <row r="33">
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="V33">
-        <v>0.7217941176470588</v>
+        <v>0.7246888888888889</v>
       </c>
     </row>
     <row r="34">
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="V34">
-        <v>0.8350823529411765</v>
+        <v>0.8372999999999999</v>
       </c>
     </row>
     <row r="35">
@@ -2967,7 +2967,7 @@
         </is>
       </c>
       <c r="V35">
-        <v>0.7387117647058824</v>
+        <v>0.7410555555555556</v>
       </c>
     </row>
     <row r="36">
@@ -3041,7 +3041,7 @@
         </is>
       </c>
       <c r="V36">
-        <v>0.6837941176470589</v>
+        <v>0.6855722222222222</v>
       </c>
     </row>
     <row r="37">
@@ -3109,7 +3109,7 @@
         </is>
       </c>
       <c r="V37">
-        <v>0.6557733333333333</v>
+        <v>0.65723125</v>
       </c>
     </row>
     <row r="38">
@@ -3183,7 +3183,7 @@
         </is>
       </c>
       <c r="V38">
-        <v>0.7709588235294118</v>
+        <v>0.7731111111111111</v>
       </c>
     </row>
     <row r="39">
@@ -3257,7 +3257,7 @@
         </is>
       </c>
       <c r="V39">
-        <v>0.6795176470588236</v>
+        <v>0.6807166666666666</v>
       </c>
     </row>
     <row r="40">
@@ -3331,7 +3331,7 @@
         </is>
       </c>
       <c r="V40">
-        <v>0.6819117647058823</v>
+        <v>0.6836777777777777</v>
       </c>
     </row>
     <row r="41">
@@ -3405,7 +3405,7 @@
         </is>
       </c>
       <c r="V41">
-        <v>0.6439823529411765</v>
+        <v>0.6469166666666667</v>
       </c>
     </row>
     <row r="42">
@@ -3479,7 +3479,7 @@
         </is>
       </c>
       <c r="V42">
-        <v>0.694535294117647</v>
+        <v>0.6963055555555555</v>
       </c>
     </row>
     <row r="43">
@@ -3553,7 +3553,7 @@
         </is>
       </c>
       <c r="V43">
-        <v>0.6774058823529412</v>
+        <v>0.6778888888888889</v>
       </c>
     </row>
     <row r="44">
@@ -3627,7 +3627,7 @@
         </is>
       </c>
       <c r="V44">
-        <v>0.8571470588235294</v>
+        <v>0.8614777777777778</v>
       </c>
     </row>
     <row r="45">
@@ -3701,7 +3701,7 @@
         </is>
       </c>
       <c r="V45">
-        <v>0.6376823529411765</v>
+        <v>0.6378555555555555</v>
       </c>
     </row>
     <row r="46">
@@ -3775,7 +3775,7 @@
         </is>
       </c>
       <c r="V46">
-        <v>0.6738294117647059</v>
+        <v>0.6745277777777777</v>
       </c>
     </row>
     <row r="47">
@@ -3849,7 +3849,7 @@
         </is>
       </c>
       <c r="V47">
-        <v>0.5855176470588235</v>
+        <v>0.5851388888888889</v>
       </c>
     </row>
     <row r="48">
@@ -3923,7 +3923,7 @@
         </is>
       </c>
       <c r="V48">
-        <v>0.781964705882353</v>
+        <v>0.7830833333333334</v>
       </c>
     </row>
     <row r="49">
@@ -3997,7 +3997,7 @@
         </is>
       </c>
       <c r="V49">
-        <v>0.7066</v>
+        <v>0.7061555555555555</v>
       </c>
     </row>
     <row r="50">
@@ -4071,7 +4071,7 @@
         </is>
       </c>
       <c r="V50">
-        <v>0.6919647058823529</v>
+        <v>0.6925944444444444</v>
       </c>
     </row>
     <row r="51">
@@ -4145,7 +4145,7 @@
         </is>
       </c>
       <c r="V51">
-        <v>0.7174294117647059</v>
+        <v>0.7196722222222223</v>
       </c>
     </row>
     <row r="52">
@@ -4219,7 +4219,7 @@
         </is>
       </c>
       <c r="V52">
-        <v>0.6528529411764706</v>
+        <v>0.6534166666666666</v>
       </c>
     </row>
     <row r="53">
@@ -4293,7 +4293,7 @@
         </is>
       </c>
       <c r="V53">
-        <v>0.7107529411764706</v>
+        <v>0.7107333333333333</v>
       </c>
     </row>
     <row r="54">
@@ -4367,7 +4367,7 @@
         </is>
       </c>
       <c r="V54">
-        <v>0.6153529411764705</v>
+        <v>0.6173888888888889</v>
       </c>
     </row>
     <row r="55">
@@ -4441,7 +4441,7 @@
         </is>
       </c>
       <c r="V55">
-        <v>0.6825117647058824</v>
+        <v>0.6841722222222222</v>
       </c>
     </row>
     <row r="56">
@@ -4515,7 +4515,7 @@
         </is>
       </c>
       <c r="V56">
-        <v>0.6467294117647059</v>
+        <v>0.64945</v>
       </c>
     </row>
     <row r="57">
@@ -4589,7 +4589,7 @@
         </is>
       </c>
       <c r="V57">
-        <v>0.6352588235294118</v>
+        <v>0.6353</v>
       </c>
     </row>
     <row r="58">
@@ -4663,7 +4663,7 @@
         </is>
       </c>
       <c r="V58">
-        <v>0.6926588235294118</v>
+        <v>0.6930499999999999</v>
       </c>
     </row>
     <row r="59">
@@ -4737,7 +4737,7 @@
         </is>
       </c>
       <c r="V59">
-        <v>0.7199058823529412</v>
+        <v>0.7182999999999999</v>
       </c>
     </row>
     <row r="60">
@@ -4811,7 +4811,7 @@
         </is>
       </c>
       <c r="V60">
-        <v>0.7554529411764705</v>
+        <v>0.75645</v>
       </c>
     </row>
     <row r="61">
@@ -4885,7 +4885,7 @@
         </is>
       </c>
       <c r="V61">
-        <v>0.7406</v>
+        <v>0.7435388888888889</v>
       </c>
     </row>
     <row r="62">
@@ -4959,7 +4959,7 @@
         </is>
       </c>
       <c r="V62">
-        <v>0.717764705882353</v>
+        <v>0.7192333333333333</v>
       </c>
     </row>
     <row r="63">
@@ -5033,7 +5033,7 @@
         </is>
       </c>
       <c r="V63">
-        <v>0.6943941176470588</v>
+        <v>0.6958</v>
       </c>
     </row>
     <row r="64">
@@ -5178,7 +5178,7 @@
         </is>
       </c>
       <c r="V65">
-        <v>0.6604764705882353</v>
+        <v>0.6608833333333334</v>
       </c>
     </row>
     <row r="66">
@@ -5252,7 +5252,7 @@
         </is>
       </c>
       <c r="V66">
-        <v>0.592</v>
+        <v>0.5926722222222223</v>
       </c>
     </row>
     <row r="67">
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="V67">
-        <v>0.6765117647058824</v>
+        <v>0.6790888888888889</v>
       </c>
     </row>
     <row r="68">
@@ -5465,7 +5465,7 @@
         </is>
       </c>
       <c r="V69">
-        <v>0.658235294117647</v>
+        <v>0.6596388888888889</v>
       </c>
     </row>
     <row r="70">
@@ -5539,7 +5539,7 @@
         </is>
       </c>
       <c r="V70">
-        <v>0.6946058823529412</v>
+        <v>0.6986666666666667</v>
       </c>
     </row>
     <row r="71">
@@ -5613,7 +5613,7 @@
         </is>
       </c>
       <c r="V71">
-        <v>0.7088470588235294</v>
+        <v>0.7086277777777777</v>
       </c>
     </row>
     <row r="72">
@@ -5687,7 +5687,7 @@
         </is>
       </c>
       <c r="V72">
-        <v>0.7353235294117647</v>
+        <v>0.7384000000000001</v>
       </c>
     </row>
     <row r="73">
@@ -5761,7 +5761,7 @@
         </is>
       </c>
       <c r="V73">
-        <v>0.5940764705882353</v>
+        <v>0.5959388888888889</v>
       </c>
     </row>
     <row r="74">
@@ -5830,7 +5830,7 @@
         <v>0.8045</v>
       </c>
       <c r="V74">
-        <v>0.7468588235294118</v>
+        <v>0.7500611111111111</v>
       </c>
     </row>
     <row r="75">
@@ -5904,7 +5904,7 @@
         </is>
       </c>
       <c r="V75">
-        <v>0.6317647058823529</v>
+        <v>0.6335444444444445</v>
       </c>
     </row>
     <row r="76">
@@ -5978,7 +5978,7 @@
         </is>
       </c>
       <c r="V76">
-        <v>0.7530588235294118</v>
+        <v>0.75425</v>
       </c>
     </row>
     <row r="77">
@@ -6052,7 +6052,7 @@
         </is>
       </c>
       <c r="V77">
-        <v>0.7929352941176471</v>
+        <v>0.7952555555555556</v>
       </c>
     </row>
     <row r="78">
@@ -6126,7 +6126,7 @@
         </is>
       </c>
       <c r="V78">
-        <v>0.7558294117647059</v>
+        <v>0.7589166666666667</v>
       </c>
     </row>
     <row r="79">
@@ -6200,7 +6200,7 @@
         </is>
       </c>
       <c r="V79">
-        <v>0.6287882352941176</v>
+        <v>0.6299722222222223</v>
       </c>
     </row>
     <row r="80">
@@ -6274,7 +6274,7 @@
         </is>
       </c>
       <c r="V80">
-        <v>0.8366823529411764</v>
+        <v>0.8388055555555556</v>
       </c>
     </row>
     <row r="81">
@@ -6348,7 +6348,7 @@
         </is>
       </c>
       <c r="V81">
-        <v>0.5538999999999999</v>
+        <v>0.5547666666666666</v>
       </c>
     </row>
     <row r="82">
@@ -6422,7 +6422,7 @@
         </is>
       </c>
       <c r="V82">
-        <v>0.7165705882352942</v>
+        <v>0.7179888888888889</v>
       </c>
     </row>
     <row r="83">
@@ -6496,7 +6496,7 @@
         </is>
       </c>
       <c r="V83">
-        <v>0.6777058823529412</v>
+        <v>0.6793055555555555</v>
       </c>
     </row>
     <row r="84">
@@ -6570,7 +6570,7 @@
         </is>
       </c>
       <c r="V84">
-        <v>0.7013058823529412</v>
+        <v>0.7042944444444444</v>
       </c>
     </row>
     <row r="85">
@@ -6644,7 +6644,7 @@
         </is>
       </c>
       <c r="V85">
-        <v>0.7769058823529412</v>
+        <v>0.7770222222222223</v>
       </c>
     </row>
     <row r="86">
@@ -6718,7 +6718,7 @@
         </is>
       </c>
       <c r="V86">
-        <v>0.7085176470588235</v>
+        <v>0.7102666666666666</v>
       </c>
     </row>
     <row r="87">
@@ -6792,7 +6792,7 @@
         </is>
       </c>
       <c r="V87">
-        <v>0.7263294117647059</v>
+        <v>0.7297166666666667</v>
       </c>
     </row>
     <row r="88">
@@ -6866,7 +6866,7 @@
         </is>
       </c>
       <c r="V88">
-        <v>0.6927647058823529</v>
+        <v>0.6941055555555555</v>
       </c>
     </row>
     <row r="89">
@@ -7005,7 +7005,7 @@
         </is>
       </c>
       <c r="V90">
-        <v>0.5857470588235294</v>
+        <v>0.5891222222222222</v>
       </c>
     </row>
     <row r="91">
@@ -7079,7 +7079,7 @@
         </is>
       </c>
       <c r="V91">
-        <v>0.6992411764705883</v>
+        <v>0.7017055555555556</v>
       </c>
     </row>
     <row r="92">
@@ -7153,7 +7153,7 @@
         </is>
       </c>
       <c r="V92">
-        <v>0.6903294117647059</v>
+        <v>0.6925888888888889</v>
       </c>
     </row>
     <row r="93">
@@ -7227,7 +7227,7 @@
         </is>
       </c>
       <c r="V93">
-        <v>0.7348235294117647</v>
+        <v>0.7365333333333334</v>
       </c>
     </row>
     <row r="94">
@@ -7301,7 +7301,7 @@
         </is>
       </c>
       <c r="V94">
-        <v>0.7555705882352941</v>
+        <v>0.7572277777777778</v>
       </c>
     </row>
     <row r="95">
@@ -7369,7 +7369,7 @@
         </is>
       </c>
       <c r="V95">
-        <v>0.6941733333333333</v>
+        <v>0.69700625</v>
       </c>
     </row>
     <row r="96">
@@ -7443,7 +7443,7 @@
         </is>
       </c>
       <c r="V96">
-        <v>0.7512882352941177</v>
+        <v>0.7538555555555555</v>
       </c>
     </row>
     <row r="97">
@@ -7517,7 +7517,7 @@
         </is>
       </c>
       <c r="V97">
-        <v>0.6920999999999999</v>
+        <v>0.6949833333333333</v>
       </c>
     </row>
     <row r="98">
@@ -7591,7 +7591,7 @@
         </is>
       </c>
       <c r="V98">
-        <v>0.8158705882352941</v>
+        <v>0.8158555555555556</v>
       </c>
     </row>
     <row r="99">
@@ -7665,7 +7665,7 @@
         </is>
       </c>
       <c r="V99">
-        <v>0.7609705882352942</v>
+        <v>0.7623</v>
       </c>
     </row>
     <row r="100">
@@ -7739,7 +7739,7 @@
         </is>
       </c>
       <c r="V100">
-        <v>0.6970705882352941</v>
+        <v>0.69835</v>
       </c>
     </row>
     <row r="101">
@@ -7872,7 +7872,7 @@
         </is>
       </c>
       <c r="V102">
-        <v>0.6489823529411765</v>
+        <v>0.6525333333333333</v>
       </c>
     </row>
     <row r="103">
@@ -7940,7 +7940,7 @@
         </is>
       </c>
       <c r="V103">
-        <v>0.6356666666666667</v>
+        <v>0.63766875</v>
       </c>
     </row>
     <row r="104">
@@ -8014,7 +8014,7 @@
         </is>
       </c>
       <c r="V104">
-        <v>0.6111941176470588</v>
+        <v>0.6130555555555556</v>
       </c>
     </row>
     <row r="105">
@@ -8088,7 +8088,7 @@
         </is>
       </c>
       <c r="V105">
-        <v>0.7082529411764706</v>
+        <v>0.7081055555555555</v>
       </c>
     </row>
     <row r="106">
@@ -8162,7 +8162,7 @@
         </is>
       </c>
       <c r="V106">
-        <v>0.6980647058823529</v>
+        <v>0.6994055555555555</v>
       </c>
     </row>
     <row r="107">
@@ -8236,7 +8236,7 @@
         </is>
       </c>
       <c r="V107">
-        <v>0.7017529411764706</v>
+        <v>0.7031499999999999</v>
       </c>
     </row>
     <row r="108">
@@ -8310,7 +8310,7 @@
         </is>
       </c>
       <c r="V108">
-        <v>0.6043352941176471</v>
+        <v>0.6057055555555556</v>
       </c>
     </row>
     <row r="109">
@@ -8384,7 +8384,7 @@
         </is>
       </c>
       <c r="V109">
-        <v>0.7554823529411765</v>
+        <v>0.7573611111111112</v>
       </c>
     </row>
     <row r="110">
@@ -8458,7 +8458,7 @@
         </is>
       </c>
       <c r="V110">
-        <v>0.7057764705882352</v>
+        <v>0.7073611111111111</v>
       </c>
     </row>
     <row r="111">
@@ -8532,7 +8532,7 @@
         </is>
       </c>
       <c r="V111">
-        <v>0.7323294117647059</v>
+        <v>0.7331166666666666</v>
       </c>
     </row>
     <row r="112">
@@ -8606,7 +8606,7 @@
         </is>
       </c>
       <c r="V112">
-        <v>0.6324764705882353</v>
+        <v>0.6340777777777777</v>
       </c>
     </row>
     <row r="113">
@@ -8680,7 +8680,7 @@
         </is>
       </c>
       <c r="V113">
-        <v>0.6924411764705882</v>
+        <v>0.6937055555555556</v>
       </c>
     </row>
     <row r="114">
@@ -8875,7 +8875,7 @@
         </is>
       </c>
       <c r="V116">
-        <v>0.6570928571428571</v>
+        <v>0.6597466666666667</v>
       </c>
     </row>
     <row r="117">
@@ -8946,7 +8946,7 @@
         </is>
       </c>
       <c r="V117">
-        <v>0.67406875</v>
+        <v>0.6747352941176471</v>
       </c>
     </row>
     <row r="118">
@@ -9017,7 +9017,7 @@
         </is>
       </c>
       <c r="V118">
-        <v>0.67408125</v>
+        <v>0.6768470588235294</v>
       </c>
     </row>
     <row r="119">
@@ -9088,7 +9088,7 @@
         </is>
       </c>
       <c r="V119">
-        <v>0.668125</v>
+        <v>0.6697411764705882</v>
       </c>
     </row>
     <row r="120">
@@ -9147,7 +9147,7 @@
         </is>
       </c>
       <c r="V120">
-        <v>0.7361833333333333</v>
+        <v>0.7359384615384615</v>
       </c>
     </row>
     <row r="121">
@@ -9280,7 +9280,7 @@
         </is>
       </c>
       <c r="V122">
-        <v>0.65133125</v>
+        <v>0.6502529411764706</v>
       </c>
     </row>
     <row r="123">
@@ -9351,7 +9351,7 @@
         </is>
       </c>
       <c r="V123">
-        <v>0.735175</v>
+        <v>0.7376</v>
       </c>
     </row>
     <row r="124">
@@ -9419,7 +9419,7 @@
         </is>
       </c>
       <c r="V124">
-        <v>0.602</v>
+        <v>0.60365</v>
       </c>
     </row>
     <row r="125">
@@ -9490,7 +9490,7 @@
         </is>
       </c>
       <c r="V125">
-        <v>0.6221375</v>
+        <v>0.6231882352941176</v>
       </c>
     </row>
     <row r="126">
@@ -9561,7 +9561,7 @@
         </is>
       </c>
       <c r="V126">
-        <v>0.69135625</v>
+        <v>0.6927235294117647</v>
       </c>
     </row>
     <row r="127">
@@ -9632,7 +9632,7 @@
         </is>
       </c>
       <c r="V127">
-        <v>0.679875</v>
+        <v>0.683364705882353</v>
       </c>
     </row>
     <row r="128">
@@ -9765,7 +9765,7 @@
         </is>
       </c>
       <c r="V129">
-        <v>0.6603625</v>
+        <v>0.6611058823529412</v>
       </c>
     </row>
     <row r="130">
@@ -9833,7 +9833,7 @@
         </is>
       </c>
       <c r="V130">
-        <v>0.7398066666666666</v>
+        <v>0.7418625</v>
       </c>
     </row>
     <row r="131">
@@ -9901,7 +9901,7 @@
         </is>
       </c>
       <c r="V131">
-        <v>0.67408</v>
+        <v>0.6746875</v>
       </c>
     </row>
     <row r="132">
@@ -10019,7 +10019,7 @@
         </is>
       </c>
       <c r="V133">
-        <v>0.6468692307692308</v>
+        <v>0.6465071428571428</v>
       </c>
     </row>
     <row r="134">
@@ -10084,7 +10084,7 @@
         </is>
       </c>
       <c r="V134">
-        <v>0.6754071428571429</v>
+        <v>0.6756733333333333</v>
       </c>
     </row>
     <row r="135">
@@ -10146,7 +10146,7 @@
         </is>
       </c>
       <c r="V135">
-        <v>0.6046307692307692</v>
+        <v>0.6082428571428572</v>
       </c>
     </row>
     <row r="136">
@@ -10208,7 +10208,7 @@
         </is>
       </c>
       <c r="V136">
-        <v>0.6085615384615385</v>
+        <v>0.6102071428571428</v>
       </c>
     </row>
     <row r="137">
@@ -10267,7 +10267,7 @@
         </is>
       </c>
       <c r="V137">
-        <v>0.7518166666666667</v>
+        <v>0.7522</v>
       </c>
     </row>
     <row r="138">
@@ -10323,7 +10323,7 @@
         </is>
       </c>
       <c r="V138">
-        <v>0.7195727272727273</v>
+        <v>0.7225333333333334</v>
       </c>
     </row>
     <row r="139">
@@ -10370,7 +10370,7 @@
         </is>
       </c>
       <c r="V139">
-        <v>0.6741</v>
+        <v>0.6773666666666667</v>
       </c>
     </row>
     <row r="140">
@@ -10426,7 +10426,7 @@
         </is>
       </c>
       <c r="V140">
-        <v>0.7342181818181818</v>
+        <v>0.7379416666666667</v>
       </c>
     </row>
     <row r="141">
@@ -10479,7 +10479,7 @@
         </is>
       </c>
       <c r="V141">
-        <v>0.64579</v>
+        <v>0.6462636363636364</v>
       </c>
     </row>
     <row r="142">
@@ -10532,7 +10532,7 @@
         </is>
       </c>
       <c r="V142">
-        <v>0.72388</v>
+        <v>0.7217363636363636</v>
       </c>
     </row>
     <row r="143">
@@ -10582,7 +10582,7 @@
         </is>
       </c>
       <c r="V143">
-        <v>0.6378555555555555</v>
+        <v>0.63418</v>
       </c>
     </row>
     <row r="144">
@@ -10632,7 +10632,7 @@
         </is>
       </c>
       <c r="V144">
-        <v>0.6830111111111111</v>
+        <v>0.69007</v>
       </c>
     </row>
     <row r="145">
@@ -10682,7 +10682,7 @@
         </is>
       </c>
       <c r="V145">
-        <v>0.7056111111111111</v>
+        <v>0.70688</v>
       </c>
     </row>
     <row r="146">
@@ -10732,7 +10732,7 @@
         </is>
       </c>
       <c r="V146">
-        <v>0.8007555555555556</v>
+        <v>0.79634</v>
       </c>
     </row>
     <row r="147">
@@ -10776,7 +10776,7 @@
         </is>
       </c>
       <c r="V147">
-        <v>0.7046285714285714</v>
+        <v>0.7052875</v>
       </c>
     </row>
     <row r="148">
@@ -10852,7 +10852,7 @@
         </is>
       </c>
       <c r="V149">
-        <v>0.58458</v>
+        <v>0.5887</v>
       </c>
     </row>
     <row r="150">
@@ -10919,7 +10919,7 @@
         </is>
       </c>
       <c r="V151">
-        <v>0.6645800000000001</v>
+        <v>0.6717500000000001</v>
       </c>
     </row>
     <row r="152">
@@ -10957,7 +10957,7 @@
         </is>
       </c>
       <c r="V152">
-        <v>0.66196</v>
+        <v>0.6699666666666666</v>
       </c>
     </row>
     <row r="153">
@@ -10992,7 +10992,7 @@
         </is>
       </c>
       <c r="V153">
-        <v>0.6525000000000001</v>
+        <v>0.65666</v>
       </c>
     </row>
     <row r="154">
@@ -11076,7 +11076,7 @@
         </is>
       </c>
       <c r="V156">
-        <v>0.7399</v>
+        <v>0.7483</v>
       </c>
     </row>
     <row r="157">
@@ -11108,7 +11108,7 @@
         </is>
       </c>
       <c r="V157">
-        <v>0.6288333333333334</v>
+        <v>0.6284999999999999</v>
       </c>
     </row>
     <row r="158">
@@ -11137,7 +11137,7 @@
         </is>
       </c>
       <c r="V158">
-        <v>0.6475</v>
+        <v>0.6526333333333334</v>
       </c>
     </row>
     <row r="159">
@@ -11159,6 +11159,9 @@
           <t>SD</t>
         </is>
       </c>
+      <c r="V159">
+        <v>0.5679</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -11178,6 +11181,9 @@
         <is>
           <t>UZ</t>
         </is>
+      </c>
+      <c r="V160">
+        <v>0.6806</v>
       </c>
     </row>
   </sheetData>

</xml_diff>